<commit_message>
update van nieuwe eindopdracht
</commit_message>
<xml_diff>
--- a/Tabel 4 bits negate.xlsx
+++ b/Tabel 4 bits negate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pietervanengelen/Documents/QModules/computer_arch_syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{593D86AA-78CD-9D45-A72A-53F390A18988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD1BE36-BDDD-5D41-B439-4CCA1B690ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{8EF4BBC5-6694-8F41-8774-97BCE8DE0E52}"/>
+    <workbookView xWindow="27240" yWindow="5860" windowWidth="25760" windowHeight="17500" xr2:uid="{8EF4BBC5-6694-8F41-8774-97BCE8DE0E52}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>in2</t>
   </si>
@@ -66,19 +66,37 @@
   </si>
   <si>
     <t>in3 XOR in4</t>
+  </si>
+  <si>
+    <t>(b &amp;&amp; ~c &amp;&amp; ~d) || ( ~b &amp;&amp; c) || ( ~b &amp;&amp; d)</t>
+  </si>
+  <si>
+    <t>(a &amp;&amp; ~b &amp;&amp; ~c &amp;&amp; ~d) || ( ~a &amp;&amp; b) || ( ~a &amp;&amp; c) || ( ~a &amp;&amp; d)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Console"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Console"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -218,13 +236,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -232,6 +249,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -566,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F1C3B32-9C03-3C4B-B272-5719A1979612}">
-  <dimension ref="B1:N19"/>
+  <dimension ref="B1:N25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.2">
@@ -575,28 +594,28 @@
       </c>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" s="12" t="s">
+      <c r="C3" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>7</v>
       </c>
       <c r="K3" t="s">
@@ -612,7 +631,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:14" ht="18" x14ac:dyDescent="0.2">
       <c r="B4" s="1">
         <v>0</v>
       </c>
@@ -636,6 +655,12 @@
       </c>
       <c r="I4" s="3">
         <v>0</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>10</v>
       </c>
       <c r="M4" t="s">
         <v>9</v>
@@ -648,25 +673,25 @@
       <c r="B5" s="4">
         <v>0</v>
       </c>
-      <c r="C5" s="5">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5">
-        <v>0</v>
-      </c>
-      <c r="E5" s="6">
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>1</v>
       </c>
       <c r="F5" s="4">
         <v>1</v>
       </c>
-      <c r="G5" s="5">
-        <v>1</v>
-      </c>
-      <c r="H5" s="5">
-        <v>1</v>
-      </c>
-      <c r="I5" s="6">
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5">
         <v>1</v>
       </c>
     </row>
@@ -674,51 +699,51 @@
       <c r="B6" s="4">
         <v>0</v>
       </c>
-      <c r="C6" s="5">
-        <v>0</v>
-      </c>
-      <c r="D6" s="5">
-        <v>1</v>
-      </c>
-      <c r="E6" s="6">
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5">
         <v>0</v>
       </c>
       <c r="F6" s="4">
         <v>1</v>
       </c>
-      <c r="G6" s="5">
-        <v>1</v>
-      </c>
-      <c r="H6" s="5">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6">
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B7" s="7">
-        <v>0</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8">
-        <v>1</v>
-      </c>
-      <c r="E7" s="9">
-        <v>1</v>
-      </c>
-      <c r="F7" s="7">
-        <v>1</v>
-      </c>
-      <c r="G7" s="8">
-        <v>1</v>
-      </c>
-      <c r="H7" s="8">
-        <v>0</v>
-      </c>
-      <c r="I7" s="9">
+      <c r="B7" s="6">
+        <v>0</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="8">
+        <v>1</v>
+      </c>
+      <c r="F7" s="6">
+        <v>1</v>
+      </c>
+      <c r="G7" s="7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="7">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8">
         <v>1</v>
       </c>
     </row>
@@ -752,25 +777,25 @@
       <c r="B9" s="4">
         <v>0</v>
       </c>
-      <c r="C9" s="5">
-        <v>1</v>
-      </c>
-      <c r="D9" s="5">
-        <v>0</v>
-      </c>
-      <c r="E9" s="6">
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5">
         <v>1</v>
       </c>
       <c r="F9" s="4">
         <v>1</v>
       </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="5">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5">
         <v>1</v>
       </c>
     </row>
@@ -778,51 +803,51 @@
       <c r="B10" s="4">
         <v>0</v>
       </c>
-      <c r="C10" s="5">
-        <v>1</v>
-      </c>
-      <c r="D10" s="5">
-        <v>1</v>
-      </c>
-      <c r="E10" s="6">
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" s="5">
         <v>0</v>
       </c>
       <c r="F10" s="4">
         <v>1</v>
       </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="5">
-        <v>1</v>
-      </c>
-      <c r="I10" s="6">
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B11" s="7">
-        <v>0</v>
-      </c>
-      <c r="C11" s="8">
-        <v>1</v>
-      </c>
-      <c r="D11" s="8">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9">
-        <v>1</v>
-      </c>
-      <c r="F11" s="7">
-        <v>1</v>
-      </c>
-      <c r="G11" s="8">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8">
-        <v>0</v>
-      </c>
-      <c r="I11" s="9">
+      <c r="B11" s="6">
+        <v>0</v>
+      </c>
+      <c r="C11" s="7">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7">
+        <v>1</v>
+      </c>
+      <c r="E11" s="8">
+        <v>1</v>
+      </c>
+      <c r="F11" s="6">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8">
         <v>1</v>
       </c>
     </row>
@@ -856,25 +881,25 @@
       <c r="B13" s="4">
         <v>1</v>
       </c>
-      <c r="C13" s="5">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6">
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5">
         <v>1</v>
       </c>
       <c r="F13" s="4">
         <v>0</v>
       </c>
-      <c r="G13" s="5">
-        <v>1</v>
-      </c>
-      <c r="H13" s="5">
-        <v>1</v>
-      </c>
-      <c r="I13" s="6">
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13" s="5">
         <v>1</v>
       </c>
     </row>
@@ -882,51 +907,51 @@
       <c r="B14" s="4">
         <v>1</v>
       </c>
-      <c r="C14" s="5">
-        <v>0</v>
-      </c>
-      <c r="D14" s="5">
-        <v>1</v>
-      </c>
-      <c r="E14" s="6">
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" s="5">
         <v>0</v>
       </c>
       <c r="F14" s="4">
         <v>0</v>
       </c>
-      <c r="G14" s="5">
-        <v>1</v>
-      </c>
-      <c r="H14" s="5">
-        <v>1</v>
-      </c>
-      <c r="I14" s="6">
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B15" s="7">
-        <v>1</v>
-      </c>
-      <c r="C15" s="8">
-        <v>0</v>
-      </c>
-      <c r="D15" s="8">
-        <v>1</v>
-      </c>
-      <c r="E15" s="9">
-        <v>1</v>
-      </c>
-      <c r="F15" s="7">
-        <v>0</v>
-      </c>
-      <c r="G15" s="8">
-        <v>1</v>
-      </c>
-      <c r="H15" s="8">
-        <v>0</v>
-      </c>
-      <c r="I15" s="9">
+      <c r="B15" s="6">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7">
+        <v>0</v>
+      </c>
+      <c r="D15" s="7">
+        <v>1</v>
+      </c>
+      <c r="E15" s="8">
+        <v>1</v>
+      </c>
+      <c r="F15" s="6">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7">
+        <v>0</v>
+      </c>
+      <c r="I15" s="8">
         <v>1</v>
       </c>
     </row>
@@ -934,104 +959,114 @@
       <c r="B16" s="4">
         <v>1</v>
       </c>
-      <c r="C16" s="5">
-        <v>1</v>
-      </c>
-      <c r="D16" s="5">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6">
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5">
         <v>0</v>
       </c>
       <c r="F16" s="4">
         <v>0</v>
       </c>
-      <c r="G16" s="5">
-        <v>1</v>
-      </c>
-      <c r="H16" s="5">
-        <v>0</v>
-      </c>
-      <c r="I16" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B17" s="4">
         <v>1</v>
       </c>
-      <c r="C17" s="5">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6">
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5">
         <v>1</v>
       </c>
       <c r="F17" s="4">
         <v>0</v>
       </c>
-      <c r="G17" s="5">
-        <v>0</v>
-      </c>
-      <c r="H17" s="5">
-        <v>1</v>
-      </c>
-      <c r="I17" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B18" s="4">
         <v>1</v>
       </c>
-      <c r="C18" s="5">
-        <v>1</v>
-      </c>
-      <c r="D18" s="5">
-        <v>1</v>
-      </c>
-      <c r="E18" s="6">
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" s="5">
         <v>0</v>
       </c>
       <c r="F18" s="4">
         <v>0</v>
       </c>
-      <c r="G18" s="5">
-        <v>0</v>
-      </c>
-      <c r="H18" s="5">
-        <v>1</v>
-      </c>
-      <c r="I18" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="7">
-        <v>1</v>
-      </c>
-      <c r="C19" s="8">
-        <v>1</v>
-      </c>
-      <c r="D19" s="8">
-        <v>1</v>
-      </c>
-      <c r="E19" s="9">
-        <v>1</v>
-      </c>
-      <c r="F19" s="7">
-        <v>0</v>
-      </c>
-      <c r="G19" s="8">
-        <v>0</v>
-      </c>
-      <c r="H19" s="8">
-        <v>0</v>
-      </c>
-      <c r="I19" s="9">
-        <v>1</v>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B19" s="6">
+        <v>1</v>
+      </c>
+      <c r="C19" s="7">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7">
+        <v>1</v>
+      </c>
+      <c r="E19" s="8">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6">
+        <v>0</v>
+      </c>
+      <c r="G19" s="7">
+        <v>0</v>
+      </c>
+      <c r="H19" s="7">
+        <v>0</v>
+      </c>
+      <c r="I19" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" ht="18" x14ac:dyDescent="0.2">
+      <c r="L24" s="12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="K25" s="13" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>